<commit_message>
Alinha shortlist e README com a estrutura só em inglês
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QcbVoeiKE7XcrpPyAGY6tL
</commit_message>
<xml_diff>
--- a/analise/culture-and-tours-google-ads-dados.xlsx
+++ b/analise/culture-and-tours-google-ads-dados.xlsx
@@ -13,8 +13,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KP limpo'!$A$1:$T$288</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shortlist lançamento'!$A$1:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Negativas'!$A$1:$E$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Shortlist lançamento'!$A$1:$G$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Negativas'!$A$1:$E$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19826,7 +19826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -19878,7 +19878,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19909,7 +19909,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19919,7 +19919,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -19940,7 +19940,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19971,7 +19971,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -19995,14 +19995,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Alta (vigiar)</t>
+          <t>Alta, a vigiar</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -20033,7 +20033,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -20043,7 +20043,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -20057,14 +20057,14 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alta (se houver reserva no próprio dia)</t>
+          <t>Alta, se houver venda no próprio dia</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -20088,14 +20088,14 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Alta (se houver reserva no próprio dia)</t>
+          <t>Alta, se houver venda no próprio dia</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -20126,7 +20126,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -20157,7 +20157,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -20167,7 +20167,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -20188,312 +20188,108 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fado ao vivo porto</t>
+          <t>wine and fado tour porto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Frase</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1.82</v>
+          <t>Expressão</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AG2 – Vinho + Fado</t>
+          <t>EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>wine and fado tour porto</t>
+          <t>fado and wine porto</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>validar no KP</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Alta, validar no KP</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AG2 – Vinho + Fado</t>
+          <t>EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>tour vinho e fado porto</t>
+          <t>fado wine tasting porto</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>validar no KP</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Alta, validar no KP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AG2 – Vinho + Fado</t>
+          <t>EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>vinho e fado</t>
+          <t>fado tour porto</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Frase</t>
+          <t>Expressão</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>não está no ficheiro</t>
+          <t>validar no KP</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Média</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>AG2 – Vinho + Fado</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>fado and wine porto</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Frase</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>não está no ficheiro</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Alta (validar no KP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>AG2 – Vinho + Fado</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>fado wine tasting porto</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Frase</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>não está no ficheiro</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Alta (validar no KP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>AG2 – Vinho + Fado</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>fado tour porto</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Frase</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>não está no ficheiro</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Alta (validar no KP)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Reserva</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>porto fado</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Exata</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>4400</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="F19" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Reserva</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>fado no porto</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Exata</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>4400</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="F20" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Reserva</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>noite de fado porto</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Exata</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>50</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Baixa</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Reserva</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>fado no porto hoje</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Exata</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>40</v>
-      </c>
-      <c r="E22" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="F22" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Baixa</t>
+          <t>Alta, validar no KP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G22"/>
+  <autoFilter ref="A1:G15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20504,7 +20300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E137"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24162,7 +23958,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -24177,7 +23973,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Encaminhar para o AG2</t>
+          <t>Encaminhar para EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
@@ -24189,12 +23985,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>AG1 – Fado Show / Fado ao vivo</t>
+          <t>EN · Fado Show</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>vinho</t>
+          <t>tasting</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -24204,7 +24000,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Encaminhar para o AG2</t>
+          <t>Encaminhar para EN · Wine &amp; Fado</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -24213,8 +24009,35 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>EN · Fado Show</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>tour</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Phrase</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Encaminhar para EN · Wine &amp; Fado</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Rec.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E137"/>
+  <autoFilter ref="A1:E138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>